<commit_message>
Update ref  best results
</commit_message>
<xml_diff>
--- a/Homepage references.xlsx
+++ b/Homepage references.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mtsportis.sharepoint.com/sites/WorkingspaceIceland/Shared Documents/04.Input to product spec - to development/10.Measurement specification/benchmarks and references/Homepage references/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4baf5f27aaa308f5/Desktop/Measurements Github Repo/measurements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C9B8835-76DE-4971-9A34-FBC49FD6DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{2C9B8835-76DE-4971-9A34-FBC49FD6DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE9CE807-9205-4B2F-AAA0-1F21EFDA4D9A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A392E83A-501C-4FB4-93CE-0DA18CB18A6B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A392E83A-501C-4FB4-93CE-0DA18CB18A6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="1" r:id="rId1"/>
@@ -175,6 +175,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -638,7 +642,7 @@
         <v>8.3659999999999997</v>
       </c>
       <c r="L6" s="1">
-        <v>8.6259999999999994</v>
+        <v>8.1259999999999994</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -725,22 +729,22 @@
         <v>10.574999999999999</v>
       </c>
       <c r="F9" s="1">
-        <v>9.6790000000000003</v>
+        <v>9.9789999999999992</v>
       </c>
       <c r="G9" s="1">
         <v>9.5459999999999994</v>
       </c>
       <c r="H9" s="1">
-        <v>9.1170000000000009</v>
+        <v>9.4969999999999999</v>
       </c>
       <c r="I9" s="1">
         <v>9.4090000000000007</v>
       </c>
       <c r="J9" s="1">
-        <v>9.4890000000000008</v>
+        <v>9.3889999999999993</v>
       </c>
       <c r="K9" s="1">
-        <v>9.5719999999999992</v>
+        <v>9.4719999999999995</v>
       </c>
       <c r="L9" s="1">
         <v>9.3089999999999993</v>
@@ -947,13 +951,13 @@
         <v>8.8260000000000005</v>
       </c>
       <c r="J15" s="1">
-        <v>7.8760000000000003</v>
+        <v>8.31</v>
       </c>
       <c r="K15" s="1">
-        <v>8.6969999999999992</v>
+        <v>8.01</v>
       </c>
       <c r="L15" s="1">
-        <v>8.3989999999999991</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -1529,10 +1533,10 @@
         <v>10.98</v>
       </c>
       <c r="K12" s="1">
-        <v>9.89</v>
+        <v>9.99</v>
       </c>
       <c r="L12" s="1">
-        <v>9.56</v>
+        <v>9.9600000000000009</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -2248,10 +2252,10 @@
         <v>9.7100000000000009</v>
       </c>
       <c r="K13" s="1">
-        <v>9.4700000000000006</v>
+        <v>9.23</v>
       </c>
       <c r="L13" s="1">
-        <v>9.6300000000000008</v>
+        <v>9.1300000000000008</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -2540,6 +2544,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="95ec026b-a4ad-461a-a1d4-c6b927e959dc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="951160fc-ff5a-45f7-b050-f4bae28803d7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100100A38896A05B94AA42235B986E30978" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4bf31abf3bdff13eb8ffced64c31c2c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="95ec026b-a4ad-461a-a1d4-c6b927e959dc" xmlns:ns3="951160fc-ff5a-45f7-b050-f4bae28803d7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d5b6ee4a3c3b8aac6ba9922f122fd761" ns2:_="" ns3:_="">
     <xsd:import namespace="95ec026b-a4ad-461a-a1d4-c6b927e959dc"/>
@@ -2746,34 +2770,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="95ec026b-a4ad-461a-a1d4-c6b927e959dc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="951160fc-ff5a-45f7-b050-f4bae28803d7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ED17B6C-AB57-46A8-BFAB-081AE907A653}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD7541A-4617-41A2-8628-D1F9E91F5839}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD7541A-4617-41A2-8628-D1F9E91F5839}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E65F761-03A7-41D7-A089-3F63BCC3640B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="95ec026b-a4ad-461a-a1d4-c6b927e959dc"/>
+    <ds:schemaRef ds:uri="951160fc-ff5a-45f7-b050-f4bae28803d7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E65F761-03A7-41D7-A089-3F63BCC3640B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ED17B6C-AB57-46A8-BFAB-081AE907A653}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="95ec026b-a4ad-461a-a1d4-c6b927e959dc"/>
+    <ds:schemaRef ds:uri="951160fc-ff5a-45f7-b050-f4bae28803d7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update homepage references spreadsheet
</commit_message>
<xml_diff>
--- a/Homepage references.xlsx
+++ b/Homepage references.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4baf5f27aaa308f5/Desktop/Measurements Github Repo/measurements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{2C9B8835-76DE-4971-9A34-FBC49FD6DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5587FD16-0F35-4FC6-B18D-60EE88006A00}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{2C9B8835-76DE-4971-9A34-FBC49FD6DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B729CD4-A8F6-42D0-B053-D279B8E76604}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A392E83A-501C-4FB4-93CE-0DA18CB18A6B}"/>
+    <workbookView xWindow="7215" yWindow="3930" windowWidth="7500" windowHeight="9810" xr2:uid="{A392E83A-501C-4FB4-93CE-0DA18CB18A6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="1" r:id="rId1"/>
@@ -505,7 +505,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -869,7 +869,7 @@
         <v>23</v>
       </c>
       <c r="E13" s="1">
-        <v>13.844999999999999</v>
+        <v>13</v>
       </c>
       <c r="F13" s="1">
         <v>12.446000000000002</v>
@@ -881,16 +881,16 @@
         <v>11.154999999999998</v>
       </c>
       <c r="I13" s="1">
-        <v>11.577599999999999</v>
+        <v>10.853999999999999</v>
       </c>
       <c r="J13" s="1">
-        <v>10.880999999999998</v>
+        <v>10.276499999999999</v>
       </c>
       <c r="K13" s="1">
-        <v>10.98</v>
+        <v>10.37</v>
       </c>
       <c r="L13" s="1">
-        <v>10.521000000000001</v>
+        <v>9.9365000000000006</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -904,28 +904,28 @@
         <v>24</v>
       </c>
       <c r="E14" s="1">
-        <v>12.156000632838809</v>
+        <v>10.570435332903314</v>
       </c>
       <c r="F14" s="1">
-        <v>11.030749344776938</v>
+        <v>10.35751112185628</v>
       </c>
       <c r="G14" s="1">
-        <v>10.70361851495923</v>
+        <v>10.050346023435896</v>
       </c>
       <c r="H14" s="1">
-        <v>10.081766169748226</v>
+        <v>9.8017171094774422</v>
       </c>
       <c r="I14" s="1">
-        <v>10.248544047521285</v>
+        <v>9.4893926365937826</v>
       </c>
       <c r="J14" s="1">
-        <v>9.6455123974865149</v>
+        <v>9.1378538502503837</v>
       </c>
       <c r="K14" s="1">
-        <v>9.3518868866449232</v>
+        <v>9.1485849978048162</v>
       </c>
       <c r="L14" s="1">
-        <v>9.1785042314062117</v>
+        <v>8.7195790198359013</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -945,13 +945,13 @@
         <v>8.6741353772454346</v>
       </c>
       <c r="G15" s="1">
-        <v>8.0932399573808258</v>
+        <v>8.4451199555278187</v>
       </c>
       <c r="H15" s="1">
-        <v>7.7533737771005748</v>
+        <v>8.0764310178130998</v>
       </c>
       <c r="I15" s="1">
-        <v>7.4603356797274323</v>
+        <v>7.7711829997160748</v>
       </c>
       <c r="J15" s="1">
         <v>7.8347794911925126</v>
@@ -2964,6 +2964,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="95ec026b-a4ad-461a-a1d4-c6b927e959dc">
@@ -2972,15 +2981,6 @@
     <TaxCatchAll xmlns="951160fc-ff5a-45f7-b050-f4bae28803d7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3003,6 +3003,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD7541A-4617-41A2-8628-D1F9E91F5839}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E65F761-03A7-41D7-A089-3F63BCC3640B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3011,12 +3019,4 @@
     <ds:schemaRef ds:uri="951160fc-ff5a-45f7-b050-f4bae28803d7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD7541A-4617-41A2-8628-D1F9E91F5839}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>